<commit_message>
feat: add new labels for total, general, work time total, and kilometres in TimesheetGenerator and related tests
</commit_message>
<xml_diff>
--- a/app/src/main/assets/timesheet_template.xlsx
+++ b/app/src/main/assets/timesheet_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\AndroidStudioProjects\AWTimesheet\app\src\main\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A922FB-240D-4033-ADAD-790EF5F0DA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F5CF8E-46A5-4A6E-9079-3A31890FA4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
   <si>
     <t>Day of Month</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>End date</t>
+  </si>
+  <si>
+    <t>General</t>
   </si>
 </sst>
 </file>
@@ -115,10 +118,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="170" formatCode="mm\/yyyy"/>
-    <numFmt numFmtId="171" formatCode="hh:mm"/>
-    <numFmt numFmtId="172" formatCode="[hh]:mm"/>
-    <numFmt numFmtId="173" formatCode="d\.m\.yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="mm\/yyyy"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="[hh]:mm"/>
+    <numFmt numFmtId="167" formatCode="d\.m\.yyyy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -145,7 +148,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -230,77 +233,41 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,109 +614,111 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14" t="s">
+      <c r="B1" s="8"/>
+      <c r="D1" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="8" t="s">
+      <c r="I1" s="1"/>
+      <c r="J1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="M1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="N1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="14" t="s">
+      <c r="Q1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="14" t="s">
+      <c r="R1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="S1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="T1" s="31" t="s">
+      <c r="T1" s="16" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="17">
         <f>SUM(B9,G9)</f>
         <v>0.375</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="17">
         <f>SUM(B15,E9,G15)</f>
         <v>0.39583333333333337</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="17">
         <f>SUM(E15,G21)</f>
         <v>0.25</v>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="18">
         <f>SUM(E2,F2,G2)</f>
         <v>1.0208333333333335</v>
       </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="32" t="s">
+      <c r="I2" s="12"/>
+      <c r="J2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="30">
+      <c r="K2" s="19">
         <v>1</v>
       </c>
-      <c r="L2" s="30">
+      <c r="L2" s="19">
         <v>1</v>
       </c>
-      <c r="M2" s="30">
+      <c r="M2" s="19">
         <v>0</v>
       </c>
-      <c r="N2" s="33">
+      <c r="N2" s="19">
         <v>2</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="16">
+      <c r="Q2" s="17">
         <f>SUM(B9,G9)</f>
         <v>0.375</v>
       </c>
-      <c r="R2" s="16">
+      <c r="R2" s="17">
         <f>SUM(B15,E9)</f>
         <v>0.25</v>
       </c>
-      <c r="S2" s="16">
+      <c r="S2" s="17">
         <f>SUM(G21)</f>
         <v>0.1875</v>
       </c>
@@ -759,112 +728,95 @@
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="15">
         <f>SUM(B12,G12)</f>
         <v>140</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="15">
         <f>SUM(B18,E12,G18)</f>
         <v>220</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="15">
         <f>SUM(E18,G24)</f>
         <v>240</v>
       </c>
-      <c r="H3" s="20">
+      <c r="H3" s="15">
         <f>SUM(E3,F3,G3)</f>
         <v>600</v>
       </c>
-      <c r="I3" s="18"/>
-      <c r="J3" s="34" t="s">
+      <c r="J3" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="30">
+      <c r="K3" s="19">
         <v>0</v>
       </c>
-      <c r="L3" s="30">
+      <c r="L3" s="19">
         <v>1</v>
       </c>
-      <c r="M3" s="30">
+      <c r="M3" s="19">
         <v>0</v>
       </c>
-      <c r="N3" s="33">
+      <c r="N3" s="19">
         <v>1</v>
       </c>
-      <c r="P3" s="22" t="s">
+      <c r="P3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="23">
+      <c r="Q3" s="15"/>
+      <c r="R3" s="17">
         <f>SUM(G15)</f>
         <v>0.14583333333333334</v>
       </c>
-      <c r="S3" s="23">
+      <c r="S3" s="17">
         <f>SUM(E15)</f>
         <v>6.25E-2</v>
       </c>
-      <c r="T3" s="24">
+      <c r="T3" s="17">
         <f>SUM(Q3:S3)</f>
         <v>0.20833333333333334</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="28">
+      <c r="B4" s="13">
         <v>46143</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="35" t="s">
+      <c r="D4" s="1"/>
+      <c r="J4" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="36">
+      <c r="K4" s="19">
         <v>1</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="19">
         <v>1</v>
       </c>
-      <c r="M4" s="36">
+      <c r="M4" s="19">
         <v>2</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="19">
         <v>4</v>
       </c>
-      <c r="P4" s="7"/>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="14">
         <v>46173</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="O5" s="7"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>

</xml_diff>

<commit_message>
feat: add flex time total handling and related UI updates in TimesheetGenerator
</commit_message>
<xml_diff>
--- a/app/src/main/assets/timesheet_template.xlsx
+++ b/app/src/main/assets/timesheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\AndroidStudioProjects\AWTimesheet\app\src\main\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F5CF8E-46A5-4A6E-9079-3A31890FA4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98201045-8427-4F1B-9AB0-9AC904819AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="25">
   <si>
     <t>Day of Month</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>Flex time total</t>
   </si>
 </sst>
 </file>
@@ -148,7 +151,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -171,73 +174,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -251,23 +192,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -602,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE29E80-1386-45A8-BD1E-FE65E759F17A}">
-  <dimension ref="A1:AF24"/>
+  <dimension ref="A1:AF25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.1796875" customWidth="1"/>
@@ -614,54 +546,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="D1" s="16" t="s">
+      <c r="B1" s="10"/>
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" t="s">
         <v>16</v>
       </c>
       <c r="I1" s="1"/>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" t="s">
         <v>16</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="R1" t="s">
         <v>12</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" t="s">
         <v>13</v>
       </c>
-      <c r="T1" s="16" t="s">
+      <c r="T1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -672,57 +604,57 @@
       <c r="B2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="17">
-        <f>SUM(B9,G9)</f>
+      <c r="E2" s="6">
+        <f>SUM(B10,G10)</f>
         <v>0.375</v>
       </c>
-      <c r="F2" s="17">
-        <f>SUM(B15,E9,G15)</f>
+      <c r="F2" s="6">
+        <f>SUM(B16,E10,G16)</f>
         <v>0.39583333333333337</v>
       </c>
-      <c r="G2" s="17">
-        <f>SUM(E15,G21)</f>
+      <c r="G2" s="6">
+        <f>SUM(E16,G22)</f>
         <v>0.25</v>
       </c>
-      <c r="H2" s="18">
+      <c r="H2" s="6">
         <f>SUM(E2,F2,G2)</f>
         <v>1.0208333333333335</v>
       </c>
-      <c r="I2" s="12"/>
-      <c r="J2" s="18" t="s">
+      <c r="I2" s="7"/>
+      <c r="J2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="19">
+      <c r="K2" s="8">
         <v>1</v>
       </c>
-      <c r="L2" s="19">
+      <c r="L2" s="8">
         <v>1</v>
       </c>
-      <c r="M2" s="19">
+      <c r="M2" s="8">
         <v>0</v>
       </c>
-      <c r="N2" s="19">
+      <c r="N2" s="8">
         <v>2</v>
       </c>
-      <c r="P2" s="15" t="s">
+      <c r="P2" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="17">
-        <f>SUM(B9,G9)</f>
+      <c r="Q2" s="6">
+        <f>SUM(B10,G10)</f>
         <v>0.375</v>
       </c>
-      <c r="R2" s="17">
-        <f>SUM(B15,E9)</f>
+      <c r="R2" s="6">
+        <f>SUM(B16,E10)</f>
         <v>0.25</v>
       </c>
-      <c r="S2" s="17">
-        <f>SUM(G21)</f>
+      <c r="S2" s="6">
+        <f>SUM(G22)</f>
         <v>0.1875</v>
       </c>
-      <c r="T2" s="17">
+      <c r="T2" s="6">
         <f>SUM(Q2:S2)</f>
         <v>0.8125</v>
       </c>
@@ -734,53 +666,53 @@
       <c r="B3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="15">
-        <f>SUM(B12,G12)</f>
+      <c r="E3">
+        <f>SUM(B13,G13)</f>
         <v>140</v>
       </c>
-      <c r="F3" s="15">
-        <f>SUM(B18,E12,G18)</f>
+      <c r="F3">
+        <f>SUM(B19,E13,G19)</f>
         <v>220</v>
       </c>
-      <c r="G3" s="15">
-        <f>SUM(E18,G24)</f>
+      <c r="G3">
+        <f>SUM(E19,G25)</f>
         <v>240</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3">
         <f>SUM(E3,F3,G3)</f>
         <v>600</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="19">
+      <c r="K3" s="8">
         <v>0</v>
       </c>
-      <c r="L3" s="19">
+      <c r="L3" s="8">
         <v>1</v>
       </c>
-      <c r="M3" s="19">
+      <c r="M3" s="8">
         <v>0</v>
       </c>
-      <c r="N3" s="19">
+      <c r="N3" s="8">
         <v>1</v>
       </c>
-      <c r="P3" s="15" t="s">
+      <c r="P3" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="17">
-        <f>SUM(G15)</f>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6">
+        <f>SUM(G16)</f>
         <v>0.14583333333333334</v>
       </c>
-      <c r="S3" s="17">
-        <f>SUM(E15)</f>
+      <c r="S3" s="6">
+        <f>SUM(E16)</f>
         <v>6.25E-2</v>
       </c>
-      <c r="T3" s="17">
+      <c r="T3" s="6">
         <f>SUM(Q3:S3)</f>
         <v>0.20833333333333334</v>
       </c>
@@ -789,300 +721,309 @@
       <c r="A4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="11">
         <v>46143</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="J4" s="15" t="s">
+      <c r="J4" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="19">
+      <c r="K4" s="8">
         <v>1</v>
       </c>
-      <c r="L4" s="19">
+      <c r="L4" s="8">
         <v>1</v>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="8">
         <v>2</v>
       </c>
-      <c r="N4" s="19">
+      <c r="N4" s="8">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="11">
         <v>46173</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="12">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1"/>
+      <c r="B7" s="4"/>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B8" s="3">
         <v>1</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C8" s="3">
         <v>2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D8" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E8" s="3">
         <v>4</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F8" s="3">
         <v>5</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G8" s="3">
         <v>6</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H8" s="3">
         <v>7</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I8" s="3">
         <v>8</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J8" s="3">
         <v>9</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K8" s="3">
         <v>10</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L8" s="3">
         <v>11</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M8" s="3">
         <v>12</v>
       </c>
-      <c r="N7" s="3">
+      <c r="N8" s="3">
         <v>13</v>
       </c>
-      <c r="O7" s="3">
+      <c r="O8" s="3">
         <v>14</v>
       </c>
-      <c r="P7" s="3">
+      <c r="P8" s="3">
         <v>15</v>
       </c>
-      <c r="Q7" s="3">
+      <c r="Q8" s="3">
         <v>16</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R8" s="3">
         <v>17</v>
       </c>
-      <c r="S7" s="3">
+      <c r="S8" s="3">
         <v>18</v>
       </c>
-      <c r="T7" s="3">
+      <c r="T8" s="3">
         <v>19</v>
       </c>
-      <c r="U7" s="3">
+      <c r="U8" s="3">
         <v>20</v>
       </c>
-      <c r="V7" s="3">
+      <c r="V8" s="3">
         <v>21</v>
       </c>
-      <c r="W7" s="3">
+      <c r="W8" s="3">
         <v>22</v>
       </c>
-      <c r="X7" s="3">
+      <c r="X8" s="3">
         <v>23</v>
       </c>
-      <c r="Y7" s="3">
+      <c r="Y8" s="3">
         <v>24</v>
       </c>
-      <c r="Z7" s="3">
+      <c r="Z8" s="3">
         <v>25</v>
       </c>
-      <c r="AA7" s="3">
+      <c r="AA8" s="3">
         <v>26</v>
       </c>
-      <c r="AB7" s="3">
+      <c r="AB8" s="3">
         <v>27</v>
       </c>
-      <c r="AC7" s="3">
+      <c r="AC8" s="3">
         <v>28</v>
       </c>
-      <c r="AD7" s="3">
+      <c r="AD8" s="3">
         <v>29</v>
       </c>
-      <c r="AE7" s="3">
+      <c r="AE8" s="3">
         <v>30</v>
       </c>
-      <c r="AF7" s="3">
+      <c r="AF8" s="3">
         <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="6">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="E9" s="6">
-        <v>0.1875</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0.10416666666666667</v>
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5" t="s">
-        <v>19</v>
+        <v>2</v>
+      </c>
+      <c r="B10" s="6">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.1875</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0.10416666666666667</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>10</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>10</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="F11" s="5"/>
       <c r="G11" s="5" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12">
+      <c r="B13">
         <v>70</v>
       </c>
-      <c r="E12">
+      <c r="E13">
         <v>40</v>
       </c>
-      <c r="G12">
+      <c r="G13">
         <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A14" s="1"/>
-      <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
-      <c r="B15" s="6">
-        <v>6.25E-2</v>
-      </c>
-      <c r="E15" s="6">
-        <v>6.25E-2</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0.14583333333333334</v>
+      <c r="B15" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
-      <c r="B16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>19</v>
+      <c r="B16" s="6">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E16" s="6">
+        <v>6.25E-2</v>
+      </c>
+      <c r="G16" s="6">
+        <v>0.14583333333333334</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="5" t="s">
-        <v>10</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
-      <c r="B18">
+      <c r="B18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+      <c r="B19">
         <v>90</v>
       </c>
-      <c r="E18">
+      <c r="E19">
         <v>120</v>
       </c>
-      <c r="G18">
+      <c r="G19">
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G20" s="5" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G21" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G21" s="6">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G22" s="6">
         <v>0.1875</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G22" s="5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="G23" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G24" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G24">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G25">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance TimesheetGenerator with dynamic work type handling and day of month row population
</commit_message>
<xml_diff>
--- a/app/src/main/assets/timesheet_template.xlsx
+++ b/app/src/main/assets/timesheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\AndroidStudioProjects\AWTimesheet\app\src\main\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98201045-8427-4F1B-9AB0-9AC904819AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{972F6E15-DEE0-4A94-8C7B-16B72E93B21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
   </bookViews>
@@ -178,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -194,12 +194,10 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,10 +544,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="10"/>
       <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
@@ -598,10 +595,10 @@
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="D2" t="s">
@@ -660,10 +657,10 @@
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" t="s">
         <v>11</v>
       </c>
       <c r="D3" t="s">
@@ -718,10 +715,10 @@
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="9">
         <v>46143</v>
       </c>
       <c r="D4" s="1"/>
@@ -742,19 +739,19 @@
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="9">
         <v>46173</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="7">
         <v>0</v>
       </c>
       <c r="D6" s="1"/>
@@ -763,7 +760,7 @@
       <c r="A7" s="1"/>
       <c r="B7" s="4"/>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat: simplify cell styling in TimesheetGenerator by removing style indices
</commit_message>
<xml_diff>
--- a/app/src/main/assets/timesheet_template.xlsx
+++ b/app/src/main/assets/timesheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\AndroidStudioProjects\AWTimesheet\app\src\main\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{972F6E15-DEE0-4A94-8C7B-16B72E93B21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6DCA13-5793-4617-B166-BB3C60E3EBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="26">
   <si>
     <t>Day of Month</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Flex time total</t>
+  </si>
+  <si>
+    <t>Project time</t>
   </si>
 </sst>
 </file>
@@ -178,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -188,16 +191,21 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE29E80-1386-45A8-BD1E-FE65E759F17A}">
-  <dimension ref="A1:AF25"/>
+  <dimension ref="A1:AF27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.1796875" customWidth="1"/>
@@ -604,54 +612,54 @@
       <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6">
-        <f>SUM(B10,G10)</f>
+      <c r="E2" s="5">
+        <f>SUM(B12,G12)</f>
         <v>0.375</v>
       </c>
-      <c r="F2" s="6">
-        <f>SUM(B16,E10,G16)</f>
+      <c r="F2" s="5">
+        <f>SUM(B18,E12,G18)</f>
         <v>0.39583333333333337</v>
       </c>
-      <c r="G2" s="6">
-        <f>SUM(E16,G22)</f>
+      <c r="G2" s="5">
+        <f>SUM(E18,G24)</f>
         <v>0.25</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="5">
         <f>SUM(E2,F2,G2)</f>
         <v>1.0208333333333335</v>
       </c>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7" t="s">
+      <c r="I2" s="6"/>
+      <c r="J2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="8">
+      <c r="K2" s="7">
         <v>1</v>
       </c>
-      <c r="L2" s="8">
+      <c r="L2" s="7">
         <v>1</v>
       </c>
-      <c r="M2" s="8">
+      <c r="M2" s="7">
         <v>0</v>
       </c>
-      <c r="N2" s="8">
+      <c r="N2" s="7">
         <v>2</v>
       </c>
       <c r="P2" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="6">
-        <f>SUM(B10,G10)</f>
+      <c r="Q2" s="5">
+        <f>SUM(B12,G12)</f>
         <v>0.375</v>
       </c>
-      <c r="R2" s="6">
-        <f>SUM(B16,E10)</f>
+      <c r="R2" s="5">
+        <f>SUM(B18,E12)</f>
         <v>0.25</v>
       </c>
-      <c r="S2" s="6">
-        <f>SUM(G22)</f>
+      <c r="S2" s="5">
+        <f>SUM(G24)</f>
         <v>0.1875</v>
       </c>
-      <c r="T2" s="6">
+      <c r="T2" s="5">
         <f>SUM(Q2:S2)</f>
         <v>0.8125</v>
       </c>
@@ -667,15 +675,15 @@
         <v>5</v>
       </c>
       <c r="E3">
-        <f>SUM(B13,G13)</f>
+        <f>SUM(B15,G15)</f>
         <v>140</v>
       </c>
       <c r="F3">
-        <f>SUM(B19,E13,G19)</f>
+        <f>SUM(B21,E15,G21)</f>
         <v>220</v>
       </c>
       <c r="G3">
-        <f>SUM(E19,G25)</f>
+        <f>SUM(E21,G27)</f>
         <v>240</v>
       </c>
       <c r="H3">
@@ -685,31 +693,31 @@
       <c r="J3" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="7">
         <v>0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="7">
         <v>1</v>
       </c>
-      <c r="M3" s="8">
+      <c r="M3" s="7">
         <v>0</v>
       </c>
-      <c r="N3" s="8">
+      <c r="N3" s="7">
         <v>1</v>
       </c>
       <c r="P3" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6">
-        <f>SUM(G16)</f>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5">
+        <f>SUM(G18)</f>
         <v>0.14583333333333334</v>
       </c>
-      <c r="S3" s="6">
-        <f>SUM(E16)</f>
+      <c r="S3" s="5">
+        <f>SUM(E18)</f>
         <v>6.25E-2</v>
       </c>
-      <c r="T3" s="6">
+      <c r="T3" s="5">
         <f>SUM(Q3:S3)</f>
         <v>0.20833333333333334</v>
       </c>
@@ -718,23 +726,23 @@
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>46143</v>
       </c>
       <c r="D4" s="1"/>
       <c r="J4" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="7">
         <v>1</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
         <v>1</v>
       </c>
-      <c r="M4" s="8">
+      <c r="M4" s="7">
         <v>2</v>
       </c>
-      <c r="N4" s="8">
+      <c r="N4" s="7">
         <v>4</v>
       </c>
     </row>
@@ -742,7 +750,7 @@
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>46173</v>
       </c>
       <c r="D5" s="1"/>
@@ -751,7 +759,7 @@
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>0</v>
       </c>
       <c r="D6" s="1"/>
@@ -760,7 +768,7 @@
       <c r="A7" s="1"/>
       <c r="B7" s="4"/>
     </row>
-    <row r="8" spans="1:32" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
@@ -860,167 +868,271 @@
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5" t="s">
-        <v>9</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B9" s="9">
+        <f>SUM(B12,B18)</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="9">
+        <f>SUM(E12,E18)</f>
+        <v>0.25</v>
+      </c>
+      <c r="F9" s="10"/>
+      <c r="G9" s="9">
+        <f>SUM(G12,G18,G24)</f>
+        <v>0.4375</v>
+      </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
+      <c r="Y9" s="10"/>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="10"/>
+      <c r="AB9" s="10"/>
+      <c r="AC9" s="10"/>
+      <c r="AD9" s="10"/>
+      <c r="AE9" s="10"/>
+      <c r="AF9" s="10"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="6">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="E10" s="6">
-        <v>0.1875</v>
-      </c>
-      <c r="G10" s="6">
-        <v>0.10416666666666667</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="10"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" s="10"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>10</v>
+        <v>25</v>
+      </c>
+      <c r="B12" s="5">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0.1875</v>
+      </c>
+      <c r="G12" s="5">
+        <v>0.10416666666666667</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B13">
+      <c r="B15">
         <v>70</v>
       </c>
-      <c r="E13">
+      <c r="E15">
         <v>40</v>
       </c>
-      <c r="G13">
+      <c r="G15">
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A15" s="1"/>
-      <c r="B15" s="5" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5" t="s">
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5" t="s">
+      <c r="F17" s="11"/>
+      <c r="G17" s="11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A16" s="1"/>
-      <c r="B16" s="6">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="5">
         <v>6.25E-2</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E18" s="5">
         <v>6.25E-2</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G18" s="5">
         <v>0.14583333333333334</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="1"/>
-      <c r="B17" s="5" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5" t="s">
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G19" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="1"/>
-      <c r="B18" s="5" t="s">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E20" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="G20" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="1"/>
-      <c r="B19">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21">
         <v>90</v>
       </c>
-      <c r="E19">
+      <c r="E21">
         <v>120</v>
       </c>
-      <c r="G19">
+      <c r="G21">
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G21" s="5" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G23" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G22" s="6">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="5">
         <v>0.1875</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G23" s="5" t="s">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G24" s="5" t="s">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G26" s="11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G27">
         <v>120</v>
       </c>
     </row>

</xml_diff>